<commit_message>
Second approach of recycling
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/critical_materials/excel_files/Material_intensities_energyscope.xlsx
+++ b/projects/critical_materials/excel_files/Material_intensities_energyscope.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Paolo/Documents/PdM_code/EnergyScope-Quebec/projects/critical_materials/excel_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D385D5CB-BAEC-B24F-898F-C9A781766BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B83E4A86-7D63-A142-A9F4-DA02180FA6D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="37800" windowHeight="19500" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19540" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table of content" sheetId="1" r:id="rId1"/>
@@ -6030,11 +6030,29 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6048,50 +6066,33 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6104,15 +6105,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
@@ -19066,7 +19066,7 @@
       </c>
       <c r="G24" s="9"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
         <v>1085</v>
       </c>
@@ -19087,7 +19087,7 @@
       </c>
       <c r="G25" s="9"/>
     </row>
-    <row r="26" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="9" t="s">
         <v>1085</v>
       </c>
@@ -20124,7 +20124,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="73" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="9" t="s">
         <v>1085</v>
       </c>
@@ -21750,7 +21750,7 @@
       </c>
       <c r="G147" s="9"/>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A148" s="9" t="s">
         <v>1085</v>
       </c>
@@ -22964,7 +22964,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A205" s="9" t="s">
         <v>1085</v>
       </c>
@@ -22985,7 +22985,7 @@
       </c>
       <c r="G205" s="9"/>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A206" s="9" t="s">
         <v>1085</v>
       </c>
@@ -23006,7 +23006,7 @@
       </c>
       <c r="G206" s="9"/>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A207" s="9" t="s">
         <v>1085</v>
       </c>
@@ -23029,7 +23029,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="208" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A208" s="9" t="s">
         <v>1085</v>
       </c>
@@ -24425,7 +24425,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="271" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A271" s="9" t="s">
         <v>1085</v>
       </c>
@@ -24614,7 +24614,7 @@
       </c>
       <c r="G279" s="9"/>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A280" s="9" t="s">
         <v>1085</v>
       </c>
@@ -25971,7 +25971,7 @@
         <v>1202</v>
       </c>
     </row>
-    <row r="342" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A342" s="9" t="s">
         <v>1085</v>
       </c>
@@ -25994,7 +25994,7 @@
         <v>1202</v>
       </c>
     </row>
-    <row r="343" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A343" s="9" t="s">
         <v>1085</v>
       </c>
@@ -26015,7 +26015,7 @@
       </c>
       <c r="G343" s="9"/>
     </row>
-    <row r="344" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A344" s="9" t="s">
         <v>1085</v>
       </c>
@@ -26803,7 +26803,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="380" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="380" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A380" s="9" t="s">
         <v>1085</v>
       </c>
@@ -26824,7 +26824,7 @@
       </c>
       <c r="G380" s="9"/>
     </row>
-    <row r="381" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="381" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A381" s="9" t="s">
         <v>1085</v>
       </c>
@@ -26845,7 +26845,7 @@
       </c>
       <c r="G381" s="9"/>
     </row>
-    <row r="382" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="382" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A382" s="9" t="s">
         <v>1085</v>
       </c>
@@ -26868,7 +26868,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="383" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="383" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A383" s="9" t="s">
         <v>1085</v>
       </c>
@@ -26889,7 +26889,7 @@
       </c>
       <c r="G383" s="9"/>
     </row>
-    <row r="384" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="384" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A384" s="9" t="s">
         <v>1085</v>
       </c>
@@ -30384,7 +30384,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="545" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="545" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A545" s="9" t="s">
         <v>1085</v>
       </c>
@@ -30405,7 +30405,7 @@
       </c>
       <c r="G545" s="9"/>
     </row>
-    <row r="546" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="546" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A546" s="9" t="s">
         <v>1085</v>
       </c>
@@ -30428,7 +30428,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="547" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="547" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A547" s="9" t="s">
         <v>1085</v>
       </c>
@@ -31612,7 +31612,7 @@
       </c>
       <c r="G600" s="9"/>
     </row>
-    <row r="601" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="601" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A601" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32333,7 +32333,7 @@
       </c>
       <c r="G633" s="9"/>
     </row>
-    <row r="634" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="634" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A634" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32354,7 +32354,7 @@
       </c>
       <c r="G634" s="9"/>
     </row>
-    <row r="635" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="635" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A635" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32377,7 +32377,7 @@
         <v>1147</v>
       </c>
     </row>
-    <row r="636" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="636" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A636" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32398,7 +32398,7 @@
       </c>
       <c r="G636" s="9"/>
     </row>
-    <row r="637" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="637" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A637" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32652,7 +32652,7 @@
       </c>
       <c r="G648" s="9"/>
     </row>
-    <row r="649" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="649" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A649" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32673,7 +32673,7 @@
       </c>
       <c r="G649" s="9"/>
     </row>
-    <row r="650" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="650" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A650" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32694,7 +32694,7 @@
       </c>
       <c r="G650" s="9"/>
     </row>
-    <row r="651" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="651" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A651" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32717,7 +32717,7 @@
         <v>1147</v>
       </c>
     </row>
-    <row r="652" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="652" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A652" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32738,7 +32738,7 @@
       </c>
       <c r="G652" s="9"/>
     </row>
-    <row r="653" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="653" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A653" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32759,7 +32759,7 @@
       </c>
       <c r="G653" s="9"/>
     </row>
-    <row r="654" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="654" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A654" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32780,7 +32780,7 @@
       </c>
       <c r="G654" s="9"/>
     </row>
-    <row r="655" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="655" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A655" s="9" t="s">
         <v>1085</v>
       </c>
@@ -32803,7 +32803,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="656" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="656" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A656" s="9" t="s">
         <v>1085</v>
       </c>
@@ -33237,7 +33237,7 @@
       </c>
       <c r="G675" s="9"/>
     </row>
-    <row r="676" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="676" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A676" s="9" t="s">
         <v>1085</v>
       </c>
@@ -33258,7 +33258,7 @@
       </c>
       <c r="G676" s="9"/>
     </row>
-    <row r="677" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="677" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A677" s="9" t="s">
         <v>1085</v>
       </c>
@@ -33449,7 +33449,7 @@
       </c>
       <c r="G685" s="9"/>
     </row>
-    <row r="686" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="686" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A686" s="9" t="s">
         <v>1085</v>
       </c>
@@ -33892,7 +33892,7 @@
       </c>
       <c r="G706" s="9"/>
     </row>
-    <row r="707" spans="1:7" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="707" spans="1:7" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A707" s="9" t="s">
         <v>1085</v>
       </c>
@@ -35731,7 +35731,7 @@
       </c>
       <c r="G793" s="9"/>
     </row>
-    <row r="794" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="794" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A794" s="9" t="s">
         <v>1221</v>
       </c>
@@ -35752,7 +35752,7 @@
       </c>
       <c r="G794" s="9"/>
     </row>
-    <row r="795" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="795" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A795" s="9" t="s">
         <v>1221</v>
       </c>
@@ -35773,7 +35773,7 @@
       </c>
       <c r="G795" s="9"/>
     </row>
-    <row r="796" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="796" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A796" s="9" t="s">
         <v>1221</v>
       </c>
@@ -35794,7 +35794,7 @@
       </c>
       <c r="G796" s="9"/>
     </row>
-    <row r="797" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="797" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A797" s="9" t="s">
         <v>1221</v>
       </c>
@@ -36031,7 +36031,7 @@
         <v>1229</v>
       </c>
     </row>
-    <row r="808" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="808" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A808" s="9" t="s">
         <v>1222</v>
       </c>
@@ -36094,7 +36094,7 @@
       </c>
       <c r="G810" s="9"/>
     </row>
-    <row r="811" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="811" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A811" s="9" t="s">
         <v>1222</v>
       </c>
@@ -36519,7 +36519,7 @@
       </c>
       <c r="G829" s="9"/>
     </row>
-    <row r="830" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="830" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A830" s="226" t="s">
         <v>1138</v>
       </c>
@@ -36701,9 +36701,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G837" xr:uid="{00000000-0009-0000-0000-00000C000000}">
-    <filterColumn colId="1">
+    <filterColumn colId="2">
       <filters>
-        <filter val="c-Si"/>
+        <filter val="Platinum"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -37166,7 +37166,7 @@
       <c r="B1" s="41" t="s">
         <v>1253</v>
       </c>
-      <c r="C1" s="277" t="s">
+      <c r="C1" s="283" t="s">
         <v>63</v>
       </c>
       <c r="D1" s="272"/>
@@ -37175,7 +37175,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="280" t="s">
+      <c r="A2" s="274" t="s">
         <v>1255</v>
       </c>
       <c r="B2" s="272"/>
@@ -37190,7 +37190,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="281" t="s">
+      <c r="A3" s="286" t="s">
         <v>1259</v>
       </c>
       <c r="B3" s="266"/>
@@ -37257,7 +37257,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="280" t="s">
+      <c r="A8" s="274" t="s">
         <v>1270</v>
       </c>
       <c r="B8" s="272"/>
@@ -37272,7 +37272,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="282" t="s">
+      <c r="A9" s="277" t="s">
         <v>82</v>
       </c>
       <c r="B9" s="115" t="s">
@@ -37289,7 +37289,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="274"/>
+      <c r="A10" s="278"/>
       <c r="B10" s="115" t="s">
         <v>1276</v>
       </c>
@@ -37304,8 +37304,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="274"/>
-      <c r="B11" s="276" t="s">
+      <c r="A11" s="278"/>
+      <c r="B11" s="282" t="s">
         <v>1279</v>
       </c>
       <c r="C11" s="36" t="s">
@@ -37314,23 +37314,23 @@
       <c r="D11" s="156" t="s">
         <v>1281</v>
       </c>
-      <c r="E11" s="278" t="s">
+      <c r="E11" s="284" t="s">
         <v>1282</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="275"/>
-      <c r="B12" s="275"/>
+      <c r="A12" s="279"/>
+      <c r="B12" s="279"/>
       <c r="C12" s="36" t="s">
         <v>1283</v>
       </c>
       <c r="D12" s="156" t="s">
         <v>1284</v>
       </c>
-      <c r="E12" s="275"/>
+      <c r="E12" s="279"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="282" t="s">
+      <c r="A13" s="277" t="s">
         <v>1285</v>
       </c>
       <c r="B13" s="272"/>
@@ -37345,7 +37345,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="282" t="s">
+      <c r="A14" s="277" t="s">
         <v>1289</v>
       </c>
       <c r="B14" s="272"/>
@@ -37360,7 +37360,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="282" t="s">
+      <c r="A15" s="277" t="s">
         <v>1291</v>
       </c>
       <c r="B15" s="266"/>
@@ -37388,7 +37388,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="286" t="s">
+      <c r="A17" s="281" t="s">
         <v>1296</v>
       </c>
       <c r="B17" s="266"/>
@@ -37455,7 +37455,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="283" t="s">
+      <c r="A22" s="276" t="s">
         <v>1306</v>
       </c>
       <c r="B22" s="272"/>
@@ -37470,7 +37470,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="283" t="s">
+      <c r="A23" s="276" t="s">
         <v>1309</v>
       </c>
       <c r="B23" s="272"/>
@@ -37485,10 +37485,10 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="285" t="s">
+      <c r="A24" s="275" t="s">
         <v>1312</v>
       </c>
-      <c r="B24" s="279" t="s">
+      <c r="B24" s="285" t="s">
         <v>1313</v>
       </c>
       <c r="C24" s="36" t="s">
@@ -37503,7 +37503,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="268"/>
-      <c r="B25" s="275"/>
+      <c r="B25" s="279"/>
       <c r="C25" s="36" t="s">
         <v>1317</v>
       </c>
@@ -37516,7 +37516,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="268"/>
-      <c r="B26" s="273" t="s">
+      <c r="B26" s="280" t="s">
         <v>1320</v>
       </c>
       <c r="C26" s="132" t="s">
@@ -37531,7 +37531,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="268"/>
-      <c r="B27" s="274"/>
+      <c r="B27" s="278"/>
       <c r="C27" s="9" t="s">
         <v>1161</v>
       </c>
@@ -37542,7 +37542,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="268"/>
-      <c r="B28" s="274"/>
+      <c r="B28" s="278"/>
       <c r="C28" s="132" t="s">
         <v>1100</v>
       </c>
@@ -37553,7 +37553,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="268"/>
-      <c r="B29" s="275"/>
+      <c r="B29" s="279"/>
       <c r="C29" s="9" t="s">
         <v>1155</v>
       </c>
@@ -37566,7 +37566,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="268"/>
-      <c r="B30" s="273" t="s">
+      <c r="B30" s="280" t="s">
         <v>1326</v>
       </c>
       <c r="C30" s="36" t="s">
@@ -37581,7 +37581,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="268"/>
-      <c r="B31" s="274"/>
+      <c r="B31" s="278"/>
       <c r="C31" s="36" t="s">
         <v>1117</v>
       </c>
@@ -37594,7 +37594,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="268"/>
-      <c r="B32" s="274"/>
+      <c r="B32" s="278"/>
       <c r="C32" s="36" t="s">
         <v>1191</v>
       </c>
@@ -37607,7 +37607,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="268"/>
-      <c r="B33" s="275"/>
+      <c r="B33" s="279"/>
       <c r="C33" s="9" t="s">
         <v>1155</v>
       </c>
@@ -37618,7 +37618,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="268"/>
-      <c r="B34" s="273" t="s">
+      <c r="B34" s="280" t="s">
         <v>99</v>
       </c>
       <c r="C34" s="36" t="s">
@@ -37633,7 +37633,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="131"/>
-      <c r="B35" s="274"/>
+      <c r="B35" s="278"/>
       <c r="C35" s="36" t="s">
         <v>1245</v>
       </c>
@@ -37646,7 +37646,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="131"/>
-      <c r="B36" s="274"/>
+      <c r="B36" s="278"/>
       <c r="C36" s="36" t="s">
         <v>1335</v>
       </c>
@@ -37659,7 +37659,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="131"/>
-      <c r="B37" s="274"/>
+      <c r="B37" s="278"/>
       <c r="C37" s="36" t="s">
         <v>217</v>
       </c>
@@ -37672,7 +37672,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="131"/>
-      <c r="B38" s="275"/>
+      <c r="B38" s="279"/>
       <c r="C38" s="154" t="s">
         <v>1249</v>
       </c>
@@ -37684,7 +37684,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="284" t="s">
+      <c r="A39" s="273" t="s">
         <v>85</v>
       </c>
       <c r="B39" s="266"/>
@@ -38103,6 +38103,14 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B7"/>
+    <mergeCell ref="A15:B16"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A39:B62"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A24:A34"/>
@@ -38113,15 +38121,7 @@
     <mergeCell ref="A17:B21"/>
     <mergeCell ref="B34:B38"/>
     <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B7"/>
-    <mergeCell ref="A15:B16"/>
     <mergeCell ref="B30:B33"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A23:B23"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="https://www.iea.org/data-and-statistics/data-tools/critical-minerals-data-explorer" xr:uid="{00000000-0004-0000-0E00-000000000000}"/>
@@ -38159,59 +38159,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A1" s="298" t="s">
+      <c r="A1" s="287" t="s">
         <v>1368</v>
       </c>
-      <c r="B1" s="296"/>
+      <c r="B1" s="288"/>
       <c r="C1" s="272"/>
     </row>
     <row r="2" spans="1:41" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:41" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="303" t="s">
+      <c r="A3" s="290" t="s">
         <v>1369</v>
       </c>
-      <c r="B3" s="293"/>
-      <c r="C3" s="293"/>
-      <c r="D3" s="293"/>
-      <c r="E3" s="293"/>
-      <c r="F3" s="293"/>
-      <c r="G3" s="293"/>
-      <c r="H3" s="293"/>
-      <c r="I3" s="293"/>
-      <c r="J3" s="293"/>
-      <c r="K3" s="293"/>
-      <c r="L3" s="293"/>
-      <c r="M3" s="293"/>
-      <c r="N3" s="293"/>
-      <c r="O3" s="293"/>
-      <c r="P3" s="294"/>
-      <c r="R3" s="289" t="s">
+      <c r="B3" s="291"/>
+      <c r="C3" s="291"/>
+      <c r="D3" s="291"/>
+      <c r="E3" s="291"/>
+      <c r="F3" s="291"/>
+      <c r="G3" s="291"/>
+      <c r="H3" s="291"/>
+      <c r="I3" s="291"/>
+      <c r="J3" s="291"/>
+      <c r="K3" s="291"/>
+      <c r="L3" s="291"/>
+      <c r="M3" s="291"/>
+      <c r="N3" s="291"/>
+      <c r="O3" s="291"/>
+      <c r="P3" s="292"/>
+      <c r="R3" s="303" t="s">
         <v>1085</v>
       </c>
-      <c r="S3" s="290"/>
-      <c r="T3" s="290"/>
-      <c r="U3" s="290"/>
-      <c r="V3" s="290"/>
-      <c r="W3" s="290"/>
-      <c r="X3" s="290"/>
-      <c r="Y3" s="290"/>
-      <c r="Z3" s="290"/>
-      <c r="AA3" s="290"/>
-      <c r="AB3" s="290"/>
-      <c r="AC3" s="290"/>
-      <c r="AD3" s="290"/>
-      <c r="AE3" s="290"/>
-      <c r="AF3" s="290"/>
-      <c r="AG3" s="291"/>
-      <c r="AI3" s="292" t="s">
+      <c r="S3" s="304"/>
+      <c r="T3" s="304"/>
+      <c r="U3" s="304"/>
+      <c r="V3" s="304"/>
+      <c r="W3" s="304"/>
+      <c r="X3" s="304"/>
+      <c r="Y3" s="304"/>
+      <c r="Z3" s="304"/>
+      <c r="AA3" s="304"/>
+      <c r="AB3" s="304"/>
+      <c r="AC3" s="304"/>
+      <c r="AD3" s="304"/>
+      <c r="AE3" s="304"/>
+      <c r="AF3" s="304"/>
+      <c r="AG3" s="305"/>
+      <c r="AI3" s="295" t="s">
         <v>1080</v>
       </c>
-      <c r="AJ3" s="293"/>
-      <c r="AK3" s="293"/>
-      <c r="AL3" s="293"/>
-      <c r="AM3" s="293"/>
-      <c r="AN3" s="293"/>
-      <c r="AO3" s="294"/>
+      <c r="AJ3" s="291"/>
+      <c r="AK3" s="291"/>
+      <c r="AL3" s="291"/>
+      <c r="AM3" s="291"/>
+      <c r="AN3" s="291"/>
+      <c r="AO3" s="292"/>
     </row>
     <row r="4" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="52" t="s">
@@ -38262,11 +38262,11 @@
     </row>
     <row r="5" spans="1:41" x14ac:dyDescent="0.2">
       <c r="B5" s="1"/>
-      <c r="C5" s="287" t="s">
+      <c r="C5" s="289" t="s">
         <v>1370</v>
       </c>
-      <c r="D5" s="296"/>
-      <c r="E5" s="296"/>
+      <c r="D5" s="288"/>
+      <c r="E5" s="288"/>
       <c r="F5" s="272"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
@@ -38330,11 +38330,11 @@
       <c r="O6" s="1"/>
       <c r="P6" s="55"/>
       <c r="R6" s="59"/>
-      <c r="T6" s="295" t="s">
+      <c r="T6" s="296" t="s">
         <v>1373</v>
       </c>
-      <c r="U6" s="296"/>
-      <c r="V6" s="296"/>
+      <c r="U6" s="288"/>
+      <c r="V6" s="288"/>
       <c r="W6" s="272"/>
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
@@ -38393,7 +38393,7 @@
       <c r="U7" s="297">
         <v>2050</v>
       </c>
-      <c r="V7" s="296"/>
+      <c r="V7" s="288"/>
       <c r="W7" s="272"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
@@ -38659,11 +38659,11 @@
     <row r="12" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A12" s="59"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="287" t="s">
+      <c r="C12" s="289" t="s">
         <v>1382</v>
       </c>
-      <c r="D12" s="296"/>
-      <c r="E12" s="296"/>
+      <c r="D12" s="288"/>
+      <c r="E12" s="288"/>
       <c r="F12" s="272"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -38787,12 +38787,12 @@
       <c r="P14" s="55"/>
       <c r="R14" s="59"/>
       <c r="S14" s="1"/>
-      <c r="T14" s="301" t="s">
+      <c r="T14" s="300" t="s">
         <v>1383</v>
       </c>
-      <c r="U14" s="302"/>
-      <c r="V14" s="302"/>
-      <c r="W14" s="302"/>
+      <c r="U14" s="301"/>
+      <c r="V14" s="301"/>
+      <c r="W14" s="301"/>
       <c r="X14" s="1"/>
       <c r="Y14" s="1"/>
       <c r="Z14" s="1"/>
@@ -38840,11 +38840,11 @@
       <c r="P15" s="55"/>
       <c r="R15" s="59"/>
       <c r="S15" s="1"/>
-      <c r="T15" s="300" t="s">
+      <c r="T15" s="299" t="s">
         <v>1085</v>
       </c>
-      <c r="U15" s="296"/>
-      <c r="V15" s="296"/>
+      <c r="U15" s="288"/>
+      <c r="V15" s="288"/>
       <c r="W15" s="272"/>
       <c r="X15" s="1"/>
       <c r="Y15" s="1"/>
@@ -39096,13 +39096,13 @@
     <row r="20" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A20" s="59"/>
       <c r="B20" s="1"/>
-      <c r="C20" s="304" t="s">
+      <c r="C20" s="293" t="s">
         <v>1384</v>
       </c>
-      <c r="D20" s="296"/>
-      <c r="E20" s="296"/>
-      <c r="F20" s="296"/>
-      <c r="G20" s="296"/>
+      <c r="D20" s="288"/>
+      <c r="E20" s="288"/>
+      <c r="F20" s="288"/>
+      <c r="G20" s="288"/>
       <c r="H20" s="272"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
@@ -39148,15 +39148,15 @@
     <row r="21" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A21" s="59"/>
       <c r="B21" s="1"/>
-      <c r="C21" s="287" t="s">
+      <c r="C21" s="289" t="s">
         <v>1385</v>
       </c>
       <c r="D21" s="272"/>
-      <c r="E21" s="287" t="s">
+      <c r="E21" s="289" t="s">
         <v>1386</v>
       </c>
       <c r="F21" s="272"/>
-      <c r="G21" s="287" t="s">
+      <c r="G21" s="289" t="s">
         <v>1387</v>
       </c>
       <c r="H21" s="272"/>
@@ -39783,10 +39783,10 @@
       <c r="C47" s="31"/>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A48" s="298" t="s">
+      <c r="A48" s="287" t="s">
         <v>1391</v>
       </c>
-      <c r="B48" s="296"/>
+      <c r="B48" s="288"/>
       <c r="C48" s="272"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
@@ -39797,18 +39797,18 @@
       <c r="A50" s="21" t="s">
         <v>1392</v>
       </c>
-      <c r="B50" s="299" t="s">
+      <c r="B50" s="298" t="s">
         <v>1393</v>
       </c>
-      <c r="C50" s="296"/>
-      <c r="D50" s="296"/>
-      <c r="E50" s="296"/>
-      <c r="F50" s="296"/>
-      <c r="G50" s="296"/>
+      <c r="C50" s="288"/>
+      <c r="D50" s="288"/>
+      <c r="E50" s="288"/>
+      <c r="F50" s="288"/>
+      <c r="G50" s="288"/>
       <c r="H50" s="272"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" s="277" t="s">
+      <c r="A51" s="283" t="s">
         <v>1394</v>
       </c>
       <c r="B51" s="272"/>
@@ -39939,10 +39939,10 @@
       <c r="C56" s="31"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A57" s="277" t="s">
+      <c r="A57" s="283" t="s">
         <v>1405</v>
       </c>
-      <c r="B57" s="296"/>
+      <c r="B57" s="288"/>
       <c r="C57" s="272"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
@@ -39990,7 +39990,7 @@
       <c r="C62" s="31"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A63" s="277" t="s">
+      <c r="A63" s="283" t="s">
         <v>1413</v>
       </c>
       <c r="B63" s="272"/>
@@ -40000,19 +40000,19 @@
       <c r="D63" s="35" t="s">
         <v>1415</v>
       </c>
-      <c r="E63" s="277" t="s">
+      <c r="E63" s="283" t="s">
         <v>1416</v>
       </c>
       <c r="F63" s="272"/>
       <c r="G63" s="35" t="s">
         <v>1417</v>
       </c>
-      <c r="H63" s="305" t="s">
+      <c r="H63" s="294" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A64" s="277" t="s">
+      <c r="A64" s="283" t="s">
         <v>1418</v>
       </c>
       <c r="B64" s="272"/>
@@ -40031,7 +40031,7 @@
       <c r="G64" s="35" t="s">
         <v>1398</v>
       </c>
-      <c r="H64" s="275"/>
+      <c r="H64" s="279"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="45" t="s">
@@ -40178,10 +40178,10 @@
       <c r="H70" s="1"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A71" s="298" t="s">
+      <c r="A71" s="287" t="s">
         <v>1420</v>
       </c>
-      <c r="B71" s="296"/>
+      <c r="B71" s="288"/>
       <c r="C71" s="272"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
@@ -40260,10 +40260,10 @@
       <c r="C78" s="31"/>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A79" s="277" t="s">
+      <c r="A79" s="283" t="s">
         <v>1405</v>
       </c>
-      <c r="B79" s="296"/>
+      <c r="B79" s="288"/>
       <c r="C79" s="272"/>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
@@ -40305,7 +40305,7 @@
       <c r="C83" s="31"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A84" s="288" t="s">
+      <c r="A84" s="302" t="s">
         <v>1431</v>
       </c>
       <c r="B84" s="35" t="s">
@@ -40417,14 +40417,9 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A79:C79"/>
-    <mergeCell ref="A63:B63"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="A3:P3"/>
-    <mergeCell ref="C20:H20"/>
-    <mergeCell ref="H63:H64"/>
-    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="R3:AG3"/>
+    <mergeCell ref="A51:B51"/>
     <mergeCell ref="AI3:AO3"/>
     <mergeCell ref="T6:W6"/>
     <mergeCell ref="U7:W7"/>
@@ -40439,9 +40434,14 @@
     <mergeCell ref="A48:C48"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A64:B64"/>
-    <mergeCell ref="A84:A85"/>
-    <mergeCell ref="R3:AG3"/>
-    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A79:C79"/>
+    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="H63:H64"/>
+    <mergeCell ref="E21:F21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>